<commit_message>
last updates for dell and mars
</commit_message>
<xml_diff>
--- a/005_Can_SapAriba_Dell_Performer/Data/CanSapAribaDellPerformerConfig.xlsx
+++ b/005_Can_SapAriba_Dell_Performer/Data/CanSapAribaDellPerformerConfig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\1files\uipath\projects\005_Can_SapAriba_Dell\005_Can_SapAriba_Dell_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CEA4E0-5473-4677-9286-2C7F35338659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D2CBDB-C325-47EC-8054-87BD1FF2245E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2880" yWindow="3150" windowWidth="21600" windowHeight="9930" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="92">
   <si>
     <t>Name</t>
   </si>
@@ -289,6 +289,18 @@
   </si>
   <si>
     <t>Billing Adjustment</t>
+  </si>
+  <si>
+    <t>outputFolderPath</t>
+  </si>
+  <si>
+    <t>C:\1files\uipath\can_ar_ariba\dell\invoice_reports\</t>
+  </si>
+  <si>
+    <t>customerNameSAP</t>
+  </si>
+  <si>
+    <t>Dell</t>
   </si>
 </sst>
 </file>
@@ -859,8 +871,22 @@
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A28" t="s">
+        <v>90</v>
+      </c>
+      <c r="B28" t="s">
+        <v>91</v>
+      </c>
+    </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="31" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>